<commit_message>
Add battery catalog and capacity calculation
</commit_message>
<xml_diff>
--- a/Excel/Line-Energy-Solar-Calculator-v0.5.xlsx
+++ b/Excel/Line-Energy-Solar-Calculator-v0.5.xlsx
@@ -10,8 +10,9 @@
     <sheet name="Results" sheetId="2" r:id="rId2"/>
     <sheet name="Inverters" sheetId="3" r:id="rId3"/>
     <sheet name="Panels" sheetId="4" r:id="rId4"/>
-    <sheet name="Mounting" sheetId="5" r:id="rId5"/>
-    <sheet name="MountingRules" sheetId="6" r:id="rId6"/>
+    <sheet name="Batteries" sheetId="5" r:id="rId5"/>
+    <sheet name="Mounting" sheetId="6" r:id="rId6"/>
+    <sheet name="MountingRules" sheetId="7" r:id="rId7"/>
   </sheets>
 </workbook>
 </file>
@@ -96,7 +97,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:D15"/>
+  <dimension ref="A1:D17"/>
   <sheetFormatPr defaultRowHeight="16"/>
   <cols>
     <col min="1" max="1" width="32" customWidth="1"/>
@@ -266,12 +267,12 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Roof type</t>
+          <t>Battery model</t>
         </is>
       </c>
       <c r="B9" t="inlineStr" s="4">
         <is>
-          <t>Metal tile</t>
+          <t>US5000</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
@@ -288,11 +289,11 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>Total panels</t>
+          <t>Battery quantity</t>
         </is>
       </c>
       <c r="B10" s="4">
-        <v>16</v>
+        <v>2</v>
       </c>
       <c r="C10" t="inlineStr">
         <is>
@@ -301,121 +302,166 @@
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>Used for mounting quantity calculation</t>
+          <t>Used for total battery capacity</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Panels per row</t>
-        </is>
-      </c>
-      <c r="B11" s="4">
-        <v>8</v>
+          <t>Roof type</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr" s="4">
+        <is>
+          <t>Metal tile</t>
+        </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>pcs</t>
+          <t/>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>Used for row and clamp calculation</t>
+          <t>Choose from dropdown</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>Rail stock length</t>
+          <t>Total panels</t>
         </is>
       </c>
       <c r="B12" s="4">
-        <v>4.2</v>
+        <v>16</v>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>m</t>
+          <t>pcs</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>Used for rail connector estimate</t>
+          <t>Used for mounting quantity calculation</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>Rail length per panel</t>
+          <t>Panels per row</t>
         </is>
       </c>
       <c r="B13" s="4">
-        <v>1.15</v>
+        <v>8</v>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>m</t>
+          <t>pcs</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>Starter assumption; adjust by panel orientation</t>
+          <t>Used for row and clamp calculation</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>Mounting reserve</t>
+          <t>Rail stock length</t>
         </is>
       </c>
       <c r="B14" s="4">
-        <v>10</v>
+        <v>4.2</v>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>%</t>
+          <t>m</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>Extra quantity reserve</t>
+          <t>Used for rail connector estimate</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
+          <t>Rail length per panel</t>
+        </is>
+      </c>
+      <c r="B15" s="4">
+        <v>1.15</v>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>m</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>Starter assumption; adjust by panel orientation</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>Mounting reserve</t>
+        </is>
+      </c>
+      <c r="B16" s="4">
+        <v>10</v>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>%</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>Extra quantity reserve</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
           <t>Design note</t>
         </is>
       </c>
-      <c r="B15" t="inlineStr">
+      <c r="B17" t="inlineStr">
         <is>
           <t>Starter calculation only</t>
         </is>
       </c>
-      <c r="C15" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="D15" t="inlineStr">
+      <c r="C17" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
         <is>
           <t>Verify datasheets and mounting manuals before commercial use</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <dataValidations count="3">
+  <dataValidations count="4">
     <dataValidation type="list" allowBlank="0" showInputMessage="1" sqref="B3" promptTitle="Inverter" prompt="Choose inverter model">
       <formula1>Inverters!$C$2:$C$185</formula1>
     </dataValidation>
     <dataValidation type="list" allowBlank="0" showInputMessage="1" sqref="B4" promptTitle="Panel" prompt="Choose panel model">
       <formula1>Panels!$C$2:$C$73</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="0" showInputMessage="1" sqref="B9" promptTitle="Roof type" prompt="Choose roof type">
+    <dataValidation type="list" allowBlank="0" showInputMessage="1" sqref="B9" promptTitle="Battery" prompt="Choose battery model">
+      <formula1>Batteries!$C$2:$C$25</formula1>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="0" showInputMessage="1" sqref="B11" promptTitle="Roof type" prompt="Choose roof type">
       <formula1>Metal tile,Standing seam,Trapezoidal sheet,Flat roof</formula1>
     </dataValidation>
   </dataValidations>
@@ -425,7 +471,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:D25"/>
+  <dimension ref="A1:D30"/>
   <sheetFormatPr defaultRowHeight="16"/>
   <cols>
     <col min="1" max="1" width="38" customWidth="1"/>
@@ -933,6 +979,106 @@
       <c r="D25" t="inlineStr">
         <is>
           <t>All checks must pass</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>Battery model</t>
+        </is>
+      </c>
+      <c r="B26" s="3">
+        <f>Inputs!B9</f>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="D26" t="inlineStr">
+        <is>
+          <t>From Inputs</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>Battery quantity</t>
+        </is>
+      </c>
+      <c r="B27" s="3">
+        <f>Inputs!B10</f>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>pcs</t>
+        </is>
+      </c>
+      <c r="D27" t="inlineStr">
+        <is>
+          <t>From Inputs</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>Battery nominal energy</t>
+        </is>
+      </c>
+      <c r="B28" s="3">
+        <f>INDEX(Batteries!E:E,MATCH(B26,Batteries!C:C,0))</f>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>kWh</t>
+        </is>
+      </c>
+      <c r="D28" t="inlineStr">
+        <is>
+          <t>From Batteries database</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>Total nominal battery energy</t>
+        </is>
+      </c>
+      <c r="B29" s="3">
+        <f>B27*B28</f>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>kWh</t>
+        </is>
+      </c>
+      <c r="D29" t="inlineStr">
+        <is>
+          <t>Battery energy x quantity</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>Battery compatibility note</t>
+        </is>
+      </c>
+      <c r="B30" s="3">
+        <f>INDEX(Batteries!M:M,MATCH(B26,Batteries!C:C,0))</f>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="D30" t="inlineStr">
+        <is>
+          <t>From Batteries database</t>
         </is>
       </c>
     </row>
@@ -23083,6 +23229,1821 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:O25"/>
+  <sheetFormatPr defaultRowHeight="16"/>
+  <cols>
+    <col min="1" max="1" width="18" customWidth="1"/>
+    <col min="2" max="2" width="24" customWidth="1"/>
+    <col min="3" max="3" width="34" customWidth="1"/>
+    <col min="13" max="13" width="24" customWidth="1"/>
+    <col min="15" max="15" width="70" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr" s="1">
+        <is>
+          <t>brand</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr" s="1">
+        <is>
+          <t>series</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr" s="1">
+        <is>
+          <t>model</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr" s="1">
+        <is>
+          <t>chemistry</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr" s="1">
+        <is>
+          <t>nominal_energy_kwh</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr" s="1">
+        <is>
+          <t>usable_energy_kwh</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr" s="1">
+        <is>
+          <t>nominal_voltage_v</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr" s="1">
+        <is>
+          <t>capacity_ah</t>
+        </is>
+      </c>
+      <c r="I1" t="inlineStr" s="1">
+        <is>
+          <t>cycle_life_min</t>
+        </is>
+      </c>
+      <c r="J1" t="inlineStr" s="1">
+        <is>
+          <t>cycle_life_max</t>
+        </is>
+      </c>
+      <c r="K1" t="inlineStr" s="1">
+        <is>
+          <t>communication</t>
+        </is>
+      </c>
+      <c r="L1" t="inlineStr" s="1">
+        <is>
+          <t>bms</t>
+        </is>
+      </c>
+      <c r="M1" t="inlineStr" s="1">
+        <is>
+          <t>compatibility</t>
+        </is>
+      </c>
+      <c r="N1" t="inlineStr" s="1">
+        <is>
+          <t>data_status</t>
+        </is>
+      </c>
+      <c r="O1" t="inlineStr" s="1">
+        <is>
+          <t>notes</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>Pylontech</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>US Series</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>US5000</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>LiFePO4</t>
+        </is>
+      </c>
+      <c r="E2">
+        <v>4.8</v>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="G2">
+        <v>48</v>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="I2">
+        <v>6000</v>
+      </c>
+      <c r="J2">
+        <v>8000</v>
+      </c>
+      <c r="K2" t="inlineStr">
+        <is>
+          <t>CAN/RS485</t>
+        </is>
+      </c>
+      <c r="L2" t="inlineStr">
+        <is>
+          <t>Integrated BMS</t>
+        </is>
+      </c>
+      <c r="M2" t="inlineStr">
+        <is>
+          <t>Deye compatible</t>
+        </is>
+      </c>
+      <c r="N2" t="inlineStr">
+        <is>
+          <t>seed_verify_datasheet</t>
+        </is>
+      </c>
+      <c r="O2" t="inlineStr">
+        <is>
+          <t>User-listed premium battery; verify exact usable energy and protocol settings.</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Pylontech</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>Force L2</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>Force L2</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>LiFePO4</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="I3">
+        <v>6000</v>
+      </c>
+      <c r="J3">
+        <v>8000</v>
+      </c>
+      <c r="K3" t="inlineStr">
+        <is>
+          <t>CAN/RS485</t>
+        </is>
+      </c>
+      <c r="L3" t="inlineStr">
+        <is>
+          <t>Integrated BMS</t>
+        </is>
+      </c>
+      <c r="M3" t="inlineStr">
+        <is>
+          <t>Deye compatible</t>
+        </is>
+      </c>
+      <c r="N3" t="inlineStr">
+        <is>
+          <t>model_only_needs_datasheet</t>
+        </is>
+      </c>
+      <c r="O3" t="inlineStr">
+        <is>
+          <t>User-listed premium low-voltage stack; datasheet parameters pending.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>Pylontech</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>Force H2</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>Force H2</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>LiFePO4</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="I4">
+        <v>6000</v>
+      </c>
+      <c r="J4">
+        <v>8000</v>
+      </c>
+      <c r="K4" t="inlineStr">
+        <is>
+          <t>CAN/RS485</t>
+        </is>
+      </c>
+      <c r="L4" t="inlineStr">
+        <is>
+          <t>Integrated BMS</t>
+        </is>
+      </c>
+      <c r="M4" t="inlineStr">
+        <is>
+          <t>Deye compatible</t>
+        </is>
+      </c>
+      <c r="N4" t="inlineStr">
+        <is>
+          <t>model_only_needs_datasheet</t>
+        </is>
+      </c>
+      <c r="O4" t="inlineStr">
+        <is>
+          <t>User-listed premium high-voltage stack; datasheet parameters pending.</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Dyness</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>BX Series</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>BX51100</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>LiFePO4</t>
+        </is>
+      </c>
+      <c r="E5">
+        <v>5.12</v>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="G5">
+        <v>51.2</v>
+      </c>
+      <c r="H5">
+        <v>100</v>
+      </c>
+      <c r="I5" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="J5" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="K5" t="inlineStr">
+        <is>
+          <t>CAN/RS485</t>
+        </is>
+      </c>
+      <c r="L5" t="inlineStr">
+        <is>
+          <t>Integrated BMS</t>
+        </is>
+      </c>
+      <c r="M5" t="inlineStr">
+        <is>
+          <t>Deye compatible</t>
+        </is>
+      </c>
+      <c r="N5" t="inlineStr">
+        <is>
+          <t>seed_verify_datasheet</t>
+        </is>
+      </c>
+      <c r="O5" t="inlineStr">
+        <is>
+          <t>User-listed value battery; verify exact cycle life and protocol settings.</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Dyness</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>PowerRack</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>PowerRack</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>LiFePO4</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="I6" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="J6" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="K6" t="inlineStr">
+        <is>
+          <t>CAN/RS485</t>
+        </is>
+      </c>
+      <c r="L6" t="inlineStr">
+        <is>
+          <t>Integrated BMS</t>
+        </is>
+      </c>
+      <c r="M6" t="inlineStr">
+        <is>
+          <t>Deye compatible</t>
+        </is>
+      </c>
+      <c r="N6" t="inlineStr">
+        <is>
+          <t>model_only_needs_datasheet</t>
+        </is>
+      </c>
+      <c r="O6" t="inlineStr">
+        <is>
+          <t>User-listed rack battery series; datasheet parameters pending.</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>Dyness</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>Tower</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>Tower</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>LiFePO4</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="H7" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="I7" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="J7" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="K7" t="inlineStr">
+        <is>
+          <t>CAN/RS485</t>
+        </is>
+      </c>
+      <c r="L7" t="inlineStr">
+        <is>
+          <t>Integrated BMS</t>
+        </is>
+      </c>
+      <c r="M7" t="inlineStr">
+        <is>
+          <t>Deye compatible</t>
+        </is>
+      </c>
+      <c r="N7" t="inlineStr">
+        <is>
+          <t>model_only_needs_datasheet</t>
+        </is>
+      </c>
+      <c r="O7" t="inlineStr">
+        <is>
+          <t>User-listed stack battery series; datasheet parameters pending.</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>Deye ESS</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>SE Series</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>SE-G5.1</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>LiFePO4</t>
+        </is>
+      </c>
+      <c r="E8">
+        <v>5.12</v>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="G8">
+        <v>51.2</v>
+      </c>
+      <c r="H8">
+        <v>100</v>
+      </c>
+      <c r="I8" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="J8" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="K8" t="inlineStr">
+        <is>
+          <t>CAN/RS485</t>
+        </is>
+      </c>
+      <c r="L8" t="inlineStr">
+        <is>
+          <t>Deye BMS</t>
+        </is>
+      </c>
+      <c r="M8" t="inlineStr">
+        <is>
+          <t>Deye native</t>
+        </is>
+      </c>
+      <c r="N8" t="inlineStr">
+        <is>
+          <t>seed_verify_datasheet</t>
+        </is>
+      </c>
+      <c r="O8" t="inlineStr">
+        <is>
+          <t>Deye ESS model; native protocol expected; verify datasheet.</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>Deye ESS</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>SE Series</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>SE-F5</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>LiFePO4</t>
+        </is>
+      </c>
+      <c r="E9">
+        <v>5.12</v>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="G9">
+        <v>51.2</v>
+      </c>
+      <c r="H9">
+        <v>100</v>
+      </c>
+      <c r="I9" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="J9" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="K9" t="inlineStr">
+        <is>
+          <t>CAN/RS485</t>
+        </is>
+      </c>
+      <c r="L9" t="inlineStr">
+        <is>
+          <t>Deye BMS</t>
+        </is>
+      </c>
+      <c r="M9" t="inlineStr">
+        <is>
+          <t>Deye native</t>
+        </is>
+      </c>
+      <c r="N9" t="inlineStr">
+        <is>
+          <t>model_only_needs_datasheet</t>
+        </is>
+      </c>
+      <c r="O9" t="inlineStr">
+        <is>
+          <t>Deye ESS model; datasheet parameters pending.</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>Deye ESS</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>RW Series</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>RW-F16</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>LiFePO4</t>
+        </is>
+      </c>
+      <c r="E10">
+        <v>16</v>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="G10">
+        <v>51.2</v>
+      </c>
+      <c r="H10" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="I10" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="J10" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="K10" t="inlineStr">
+        <is>
+          <t>CAN/RS485</t>
+        </is>
+      </c>
+      <c r="L10" t="inlineStr">
+        <is>
+          <t>Deye BMS</t>
+        </is>
+      </c>
+      <c r="M10" t="inlineStr">
+        <is>
+          <t>Deye native</t>
+        </is>
+      </c>
+      <c r="N10" t="inlineStr">
+        <is>
+          <t>seed_verify_datasheet</t>
+        </is>
+      </c>
+      <c r="O10" t="inlineStr">
+        <is>
+          <t>Deye ESS high-capacity model; verify exact energy and current limits.</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>Gobel Power</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>Rack/Wall</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>Gobel Power 5.12kWh 51.2V 100Ah</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>LiFePO4</t>
+        </is>
+      </c>
+      <c r="E11">
+        <v>5.12</v>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="G11">
+        <v>51.2</v>
+      </c>
+      <c r="H11">
+        <v>100</v>
+      </c>
+      <c r="I11" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="J11" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="K11" t="inlineStr">
+        <is>
+          <t>CAN/RS485</t>
+        </is>
+      </c>
+      <c r="L11" t="inlineStr">
+        <is>
+          <t>JK/PACE BMS</t>
+        </is>
+      </c>
+      <c r="M11" t="inlineStr">
+        <is>
+          <t>Deye compatible</t>
+        </is>
+      </c>
+      <c r="N11" t="inlineStr">
+        <is>
+          <t>model_only_needs_datasheet</t>
+        </is>
+      </c>
+      <c r="O11" t="inlineStr">
+        <is>
+          <t>User-listed mid-segment supplier; often EVE Grade A+ cells.</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>Gobel Power</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>Rack/Wall</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>Gobel Power 10.24kWh 51.2V 200Ah</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>LiFePO4</t>
+        </is>
+      </c>
+      <c r="E12">
+        <v>10.24</v>
+      </c>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="G12">
+        <v>51.2</v>
+      </c>
+      <c r="H12">
+        <v>200</v>
+      </c>
+      <c r="I12" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="J12" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="K12" t="inlineStr">
+        <is>
+          <t>CAN/RS485</t>
+        </is>
+      </c>
+      <c r="L12" t="inlineStr">
+        <is>
+          <t>JK/PACE BMS</t>
+        </is>
+      </c>
+      <c r="M12" t="inlineStr">
+        <is>
+          <t>Deye compatible</t>
+        </is>
+      </c>
+      <c r="N12" t="inlineStr">
+        <is>
+          <t>model_only_needs_datasheet</t>
+        </is>
+      </c>
+      <c r="O12" t="inlineStr">
+        <is>
+          <t>User-listed mid-segment supplier; datasheet parameters pending.</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>GSL Energy</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>Wall/Rack</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>GSL 5.12kWh 51.2V 100Ah</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>LiFePO4</t>
+        </is>
+      </c>
+      <c r="E13">
+        <v>5.12</v>
+      </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="G13">
+        <v>51.2</v>
+      </c>
+      <c r="H13">
+        <v>100</v>
+      </c>
+      <c r="I13" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="J13" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="K13" t="inlineStr">
+        <is>
+          <t>CAN/RS485</t>
+        </is>
+      </c>
+      <c r="L13" t="inlineStr">
+        <is>
+          <t>Integrated BMS</t>
+        </is>
+      </c>
+      <c r="M13" t="inlineStr">
+        <is>
+          <t>Deye compatible</t>
+        </is>
+      </c>
+      <c r="N13" t="inlineStr">
+        <is>
+          <t>model_only_needs_datasheet</t>
+        </is>
+      </c>
+      <c r="O13" t="inlineStr">
+        <is>
+          <t>User-listed supplier; EVE/CATL cells reported by user.</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>GSL Energy</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>Wall/Rack</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>GSL 10.24kWh 51.2V 200Ah</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>LiFePO4</t>
+        </is>
+      </c>
+      <c r="E14">
+        <v>10.24</v>
+      </c>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="G14">
+        <v>51.2</v>
+      </c>
+      <c r="H14">
+        <v>200</v>
+      </c>
+      <c r="I14" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="J14" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="K14" t="inlineStr">
+        <is>
+          <t>CAN/RS485</t>
+        </is>
+      </c>
+      <c r="L14" t="inlineStr">
+        <is>
+          <t>Integrated BMS</t>
+        </is>
+      </c>
+      <c r="M14" t="inlineStr">
+        <is>
+          <t>Deye compatible</t>
+        </is>
+      </c>
+      <c r="N14" t="inlineStr">
+        <is>
+          <t>model_only_needs_datasheet</t>
+        </is>
+      </c>
+      <c r="O14" t="inlineStr">
+        <is>
+          <t>User-listed supplier; datasheet parameters pending.</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>Felicity ESS</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>LPBA Series</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>LPBA48100-OL</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>LiFePO4</t>
+        </is>
+      </c>
+      <c r="E15">
+        <v>5.12</v>
+      </c>
+      <c r="F15" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="G15">
+        <v>51.2</v>
+      </c>
+      <c r="H15">
+        <v>100</v>
+      </c>
+      <c r="I15" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="J15" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="K15" t="inlineStr">
+        <is>
+          <t>CAN/RS485</t>
+        </is>
+      </c>
+      <c r="L15" t="inlineStr">
+        <is>
+          <t>Integrated BMS</t>
+        </is>
+      </c>
+      <c r="M15" t="inlineStr">
+        <is>
+          <t>Deye compatible</t>
+        </is>
+      </c>
+      <c r="N15" t="inlineStr">
+        <is>
+          <t>model_only_needs_datasheet</t>
+        </is>
+      </c>
+      <c r="O15" t="inlineStr">
+        <is>
+          <t>Common Felicity low-voltage model candidate; datasheet parameters pending.</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>Felicity ESS</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>LPBF Series</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>LPBF48100-M</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>LiFePO4</t>
+        </is>
+      </c>
+      <c r="E16">
+        <v>5.12</v>
+      </c>
+      <c r="F16" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="G16">
+        <v>51.2</v>
+      </c>
+      <c r="H16">
+        <v>100</v>
+      </c>
+      <c r="I16" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="J16" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="K16" t="inlineStr">
+        <is>
+          <t>CAN/RS485</t>
+        </is>
+      </c>
+      <c r="L16" t="inlineStr">
+        <is>
+          <t>Integrated BMS</t>
+        </is>
+      </c>
+      <c r="M16" t="inlineStr">
+        <is>
+          <t>Deye compatible</t>
+        </is>
+      </c>
+      <c r="N16" t="inlineStr">
+        <is>
+          <t>model_only_needs_datasheet</t>
+        </is>
+      </c>
+      <c r="O16" t="inlineStr">
+        <is>
+          <t>Common Felicity low-voltage model candidate; datasheet parameters pending.</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>HinaESS</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>Rack/Commercial</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>HinaESS 5.12kWh 51.2V 100Ah</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>LiFePO4</t>
+        </is>
+      </c>
+      <c r="E17">
+        <v>5.12</v>
+      </c>
+      <c r="F17" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="G17">
+        <v>51.2</v>
+      </c>
+      <c r="H17">
+        <v>100</v>
+      </c>
+      <c r="I17" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="J17" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="K17" t="inlineStr">
+        <is>
+          <t>CAN/RS485</t>
+        </is>
+      </c>
+      <c r="L17" t="inlineStr">
+        <is>
+          <t>Integrated BMS</t>
+        </is>
+      </c>
+      <c r="M17" t="inlineStr">
+        <is>
+          <t>Deye compatible</t>
+        </is>
+      </c>
+      <c r="N17" t="inlineStr">
+        <is>
+          <t>model_only_needs_datasheet</t>
+        </is>
+      </c>
+      <c r="O17" t="inlineStr">
+        <is>
+          <t>User-listed commercial battery supplier; datasheet parameters pending.</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>HinaESS</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>Rack/Commercial</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>HinaESS 10.24kWh 51.2V 200Ah</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>LiFePO4</t>
+        </is>
+      </c>
+      <c r="E18">
+        <v>10.24</v>
+      </c>
+      <c r="F18" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="G18">
+        <v>51.2</v>
+      </c>
+      <c r="H18">
+        <v>200</v>
+      </c>
+      <c r="I18" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="J18" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="K18" t="inlineStr">
+        <is>
+          <t>CAN/RS485</t>
+        </is>
+      </c>
+      <c r="L18" t="inlineStr">
+        <is>
+          <t>Integrated BMS</t>
+        </is>
+      </c>
+      <c r="M18" t="inlineStr">
+        <is>
+          <t>Deye compatible</t>
+        </is>
+      </c>
+      <c r="N18" t="inlineStr">
+        <is>
+          <t>model_only_needs_datasheet</t>
+        </is>
+      </c>
+      <c r="O18" t="inlineStr">
+        <is>
+          <t>User-listed commercial battery supplier; datasheet parameters pending.</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>Basen Green</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>Rack/Wall</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>Basen Green 5.12kWh 51.2V 100Ah</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>LiFePO4</t>
+        </is>
+      </c>
+      <c r="E19">
+        <v>5.12</v>
+      </c>
+      <c r="F19" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="G19">
+        <v>51.2</v>
+      </c>
+      <c r="H19">
+        <v>100</v>
+      </c>
+      <c r="I19" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="J19" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="K19" t="inlineStr">
+        <is>
+          <t>CAN/RS485</t>
+        </is>
+      </c>
+      <c r="L19" t="inlineStr">
+        <is>
+          <t>Integrated BMS</t>
+        </is>
+      </c>
+      <c r="M19" t="inlineStr">
+        <is>
+          <t>Deye compatible</t>
+        </is>
+      </c>
+      <c r="N19" t="inlineStr">
+        <is>
+          <t>model_only_needs_datasheet</t>
+        </is>
+      </c>
+      <c r="O19" t="inlineStr">
+        <is>
+          <t>OEM battery candidate; datasheet parameters pending.</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>Basen Green</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>Rack/Wall</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>Basen Green 10.24kWh 51.2V 200Ah</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>LiFePO4</t>
+        </is>
+      </c>
+      <c r="E20">
+        <v>10.24</v>
+      </c>
+      <c r="F20" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="G20">
+        <v>51.2</v>
+      </c>
+      <c r="H20">
+        <v>200</v>
+      </c>
+      <c r="I20" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="J20" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="K20" t="inlineStr">
+        <is>
+          <t>CAN/RS485</t>
+        </is>
+      </c>
+      <c r="L20" t="inlineStr">
+        <is>
+          <t>Integrated BMS</t>
+        </is>
+      </c>
+      <c r="M20" t="inlineStr">
+        <is>
+          <t>Deye compatible</t>
+        </is>
+      </c>
+      <c r="N20" t="inlineStr">
+        <is>
+          <t>model_only_needs_datasheet</t>
+        </is>
+      </c>
+      <c r="O20" t="inlineStr">
+        <is>
+          <t>OEM battery candidate; datasheet parameters pending.</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>HTE</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>Rack/Wall</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>HTE 5.12kWh 51.2V 100Ah</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>LiFePO4</t>
+        </is>
+      </c>
+      <c r="E21">
+        <v>5.12</v>
+      </c>
+      <c r="F21" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="G21">
+        <v>51.2</v>
+      </c>
+      <c r="H21">
+        <v>100</v>
+      </c>
+      <c r="I21" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="J21" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="K21" t="inlineStr">
+        <is>
+          <t>CAN/RS485</t>
+        </is>
+      </c>
+      <c r="L21" t="inlineStr">
+        <is>
+          <t>Integrated BMS</t>
+        </is>
+      </c>
+      <c r="M21" t="inlineStr">
+        <is>
+          <t>Deye compatible</t>
+        </is>
+      </c>
+      <c r="N21" t="inlineStr">
+        <is>
+          <t>model_only_needs_datasheet</t>
+        </is>
+      </c>
+      <c r="O21" t="inlineStr">
+        <is>
+          <t>OEM battery candidate; datasheet parameters pending.</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>SRNE ESS</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>Rack/Wall</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>SRNE ESS 5.12kWh 51.2V 100Ah</t>
+        </is>
+      </c>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>LiFePO4</t>
+        </is>
+      </c>
+      <c r="E22">
+        <v>5.12</v>
+      </c>
+      <c r="F22" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="G22">
+        <v>51.2</v>
+      </c>
+      <c r="H22">
+        <v>100</v>
+      </c>
+      <c r="I22" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="J22" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="K22" t="inlineStr">
+        <is>
+          <t>CAN/RS485</t>
+        </is>
+      </c>
+      <c r="L22" t="inlineStr">
+        <is>
+          <t>Integrated BMS</t>
+        </is>
+      </c>
+      <c r="M22" t="inlineStr">
+        <is>
+          <t>Deye compatible</t>
+        </is>
+      </c>
+      <c r="N22" t="inlineStr">
+        <is>
+          <t>model_only_needs_datasheet</t>
+        </is>
+      </c>
+      <c r="O22" t="inlineStr">
+        <is>
+          <t>OEM battery candidate; datasheet parameters pending.</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>Hinen</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>Rack/Wall</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>Hinen 5.12kWh 51.2V 100Ah</t>
+        </is>
+      </c>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>LiFePO4</t>
+        </is>
+      </c>
+      <c r="E23">
+        <v>5.12</v>
+      </c>
+      <c r="F23" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="G23">
+        <v>51.2</v>
+      </c>
+      <c r="H23">
+        <v>100</v>
+      </c>
+      <c r="I23" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="J23" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="K23" t="inlineStr">
+        <is>
+          <t>CAN/RS485</t>
+        </is>
+      </c>
+      <c r="L23" t="inlineStr">
+        <is>
+          <t>Integrated BMS</t>
+        </is>
+      </c>
+      <c r="M23" t="inlineStr">
+        <is>
+          <t>Deye compatible</t>
+        </is>
+      </c>
+      <c r="N23" t="inlineStr">
+        <is>
+          <t>model_only_needs_datasheet</t>
+        </is>
+      </c>
+      <c r="O23" t="inlineStr">
+        <is>
+          <t>OEM battery candidate; datasheet parameters pending.</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>Svolt ESS</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>Rack/Wall</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>Svolt ESS 5.12kWh 51.2V 100Ah</t>
+        </is>
+      </c>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t>LiFePO4</t>
+        </is>
+      </c>
+      <c r="E24">
+        <v>5.12</v>
+      </c>
+      <c r="F24" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="G24">
+        <v>51.2</v>
+      </c>
+      <c r="H24">
+        <v>100</v>
+      </c>
+      <c r="I24" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="J24" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="K24" t="inlineStr">
+        <is>
+          <t>CAN/RS485</t>
+        </is>
+      </c>
+      <c r="L24" t="inlineStr">
+        <is>
+          <t>Integrated BMS</t>
+        </is>
+      </c>
+      <c r="M24" t="inlineStr">
+        <is>
+          <t>Deye compatible</t>
+        </is>
+      </c>
+      <c r="N24" t="inlineStr">
+        <is>
+          <t>model_only_needs_datasheet</t>
+        </is>
+      </c>
+      <c r="O24" t="inlineStr">
+        <is>
+          <t>OEM battery candidate; datasheet parameters pending.</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>EVE Energy ESS</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>Rack/Wall</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>EVE Energy ESS 5.12kWh 51.2V 100Ah</t>
+        </is>
+      </c>
+      <c r="D25" t="inlineStr">
+        <is>
+          <t>LiFePO4</t>
+        </is>
+      </c>
+      <c r="E25">
+        <v>5.12</v>
+      </c>
+      <c r="F25" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="G25">
+        <v>51.2</v>
+      </c>
+      <c r="H25">
+        <v>100</v>
+      </c>
+      <c r="I25" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="J25" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="K25" t="inlineStr">
+        <is>
+          <t>CAN/RS485</t>
+        </is>
+      </c>
+      <c r="L25" t="inlineStr">
+        <is>
+          <t>Integrated BMS</t>
+        </is>
+      </c>
+      <c r="M25" t="inlineStr">
+        <is>
+          <t>Deye compatible</t>
+        </is>
+      </c>
+      <c r="N25" t="inlineStr">
+        <is>
+          <t>model_only_needs_datasheet</t>
+        </is>
+      </c>
+      <c r="O25" t="inlineStr">
+        <is>
+          <t>OEM battery candidate; datasheet parameters pending.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <autoFilter ref="A1:O25"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:D19"/>
   <sheetFormatPr defaultRowHeight="16"/>
   <cols>
@@ -23121,7 +25082,7 @@
         </is>
       </c>
       <c r="B2" s="3">
-        <f>Inputs!B9</f>
+        <f>Inputs!B11</f>
       </c>
       <c r="C2" t="inlineStr">
         <is>
@@ -23141,7 +25102,7 @@
         </is>
       </c>
       <c r="B3" s="3">
-        <f>Inputs!B10</f>
+        <f>Inputs!B12</f>
       </c>
       <c r="C3" t="inlineStr">
         <is>
@@ -23161,7 +25122,7 @@
         </is>
       </c>
       <c r="B4" s="3">
-        <f>Inputs!B11</f>
+        <f>Inputs!B13</f>
       </c>
       <c r="C4" t="inlineStr">
         <is>
@@ -23221,7 +25182,7 @@
         </is>
       </c>
       <c r="B7" s="3">
-        <f>B3*Inputs!B13*2</f>
+        <f>B3*Inputs!B15*2</f>
       </c>
       <c r="C7" t="inlineStr">
         <is>
@@ -23241,7 +25202,7 @@
         </is>
       </c>
       <c r="B8" s="3">
-        <f>MAX(0,ROUNDUP(B7/Inputs!B12,0)-B6)</f>
+        <f>MAX(0,ROUNDUP(B7/Inputs!B14,0)-B6)</f>
       </c>
       <c r="C8" t="inlineStr">
         <is>
@@ -23261,7 +25222,7 @@
         </is>
       </c>
       <c r="B9" s="3">
-        <f>Inputs!B14</f>
+        <f>Inputs!B16</f>
       </c>
       <c r="C9" t="inlineStr">
         <is>
@@ -23481,7 +25442,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:J33"/>
   <sheetFormatPr defaultRowHeight="16"/>

</xml_diff>